<commit_message>
Publish Paris_2024_OG, Szeged_2024_WC, Szeged_2022_JWCH
</commit_message>
<xml_diff>
--- a/events/Paris_2024_OG/Paris_2024_OG_Results.xlsx
+++ b/events/Paris_2024_OG/Paris_2024_OG_Results.xlsx
@@ -2212,6 +2212,11 @@
           <t>64580</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>61249</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
           <t>118986</t>
@@ -6382,6 +6387,11 @@
           <t>64580</t>
         </is>
       </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>61249</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9272,6 +9282,11 @@
           <t>64580</t>
         </is>
       </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>61249</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -24832,6 +24847,11 @@
           <t>64580</t>
         </is>
       </c>
+      <c r="S337" t="inlineStr">
+        <is>
+          <t>61249</t>
+        </is>
+      </c>
       <c r="T337" t="inlineStr">
         <is>
           <t>118986</t>
@@ -29194,6 +29214,11 @@
           <t>64580</t>
         </is>
       </c>
+      <c r="S394" t="inlineStr">
+        <is>
+          <t>61249</t>
+        </is>
+      </c>
       <c r="T394" t="inlineStr">
         <is>
           <t>118986</t>
@@ -30935,6 +30960,11 @@
           <t>64580</t>
         </is>
       </c>
+      <c r="S416" t="inlineStr">
+        <is>
+          <t>61249</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -36243,6 +36273,11 @@
       <c r="R488" t="inlineStr">
         <is>
           <t>64580</t>
+        </is>
+      </c>
+      <c r="S488" t="inlineStr">
+        <is>
+          <t>61249</t>
         </is>
       </c>
     </row>
@@ -47276,7 +47311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D232"/>
+  <dimension ref="A1:D233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52368,6 +52403,28 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>61249</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Aly</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>